<commit_message>
Backend migrated to railway
</commit_message>
<xml_diff>
--- a/backend/excel/Candidates.xlsx
+++ b/backend/excel/Candidates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1342,6 +1342,100 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kunal Srivastav</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>kunal@example.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>+91-9876543210</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Software &amp; IT</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Software &amp; IT</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Python, FastAPI, React, PyTorch, FAISS, Docker</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Docker</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>FastAPI, React, PyTorch</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>B.Tech from None</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Tech Corp</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Software Engineer, Tech Corp, Python, FastAPI, React, PyTorch, FAISS, Docker, B.Tech, Computer Science, Kunal Srivastav</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Software Engineer with experience at Tech Corp since 2022. Skilled in Python, FastAPI, React, PyTorch, FAISS, and Docker. Holds a B.Tech in Computer Science.</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>mock_resume_9.pdf</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>2026-08-11 15:14:38</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>